<commit_message>
Lista de usuarios completa 👍
Está horrible, pero es funcional
</commit_message>
<xml_diff>
--- a/app/assets/Copia de BASE DE TIENDAS.xlsx
+++ b/app/assets/Copia de BASE DE TIENDAS.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A5C1E52-33B1-4E5C-B7FC-3394A941F797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7915944C-D018-46BF-876E-B408E9417B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="14496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CBT" sheetId="1" r:id="rId1"/>
@@ -13,6 +13,9 @@
     <sheet name="CORREOS TDAS-SUPERVISORES " sheetId="3" r:id="rId3"/>
     <sheet name="CORREOS DE AUTORIZACIONES " sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CBT!$G$1:$M$317</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -31,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8184" uniqueCount="1971">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8187" uniqueCount="1971">
   <si>
     <t>TDA</t>
   </si>
@@ -5950,10 +5953,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -6299,10 +6301,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -6516,20 +6518,14 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="16" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -19655,10 +19651,10 @@
       <c r="A312" s="8" t="s">
         <v>1732</v>
       </c>
-      <c r="B312" s="86" t="s">
+      <c r="B312" s="82" t="s">
         <v>1969</v>
       </c>
-      <c r="C312" s="87" t="s">
+      <c r="C312" s="84" t="s">
         <v>1970</v>
       </c>
       <c r="D312" s="39" t="s">
@@ -19694,10 +19690,10 @@
       <c r="A313" s="8" t="s">
         <v>1735</v>
       </c>
-      <c r="B313" s="84" t="s">
+      <c r="B313" s="83" t="s">
         <v>1736</v>
       </c>
-      <c r="C313" s="85" t="s">
+      <c r="C313" s="84" t="s">
         <v>1967</v>
       </c>
       <c r="D313" s="39" t="s">
@@ -19800,6 +19796,9 @@
       <c r="L315" t="s">
         <v>247</v>
       </c>
+      <c r="M315" t="s">
+        <v>1750</v>
+      </c>
     </row>
     <row r="316" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
@@ -19829,6 +19828,9 @@
       <c r="L316" t="s">
         <v>247</v>
       </c>
+      <c r="M316" t="s">
+        <v>1754</v>
+      </c>
     </row>
     <row r="317" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
@@ -19858,9 +19860,12 @@
       <c r="L317" t="s">
         <v>247</v>
       </c>
+      <c r="M317" t="s">
+        <v>1758</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="G1:M314" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="G1:M317" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="H2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="K2" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -41240,7 +41245,7 @@
       <c r="B79" s="64" t="s">
         <v>1937</v>
       </c>
-      <c r="C79" s="83" t="s">
+      <c r="C79" s="85" t="s">
         <v>1938</v>
       </c>
       <c r="D79" s="77" t="s">
@@ -41260,7 +41265,7 @@
       <c r="B80" s="64" t="s">
         <v>1941</v>
       </c>
-      <c r="C80" s="83"/>
+      <c r="C80" s="85"/>
       <c r="D80" s="77" t="s">
         <v>48</v>
       </c>
@@ -41278,7 +41283,7 @@
       <c r="B81" s="64" t="s">
         <v>1944</v>
       </c>
-      <c r="C81" s="83"/>
+      <c r="C81" s="85"/>
       <c r="D81" s="77" t="s">
         <v>57</v>
       </c>
@@ -41296,7 +41301,7 @@
       <c r="B82" s="64" t="s">
         <v>1947</v>
       </c>
-      <c r="C82" s="83"/>
+      <c r="C82" s="85"/>
       <c r="D82" s="77" t="s">
         <v>128</v>
       </c>
@@ -41314,7 +41319,7 @@
       <c r="B83" s="64" t="s">
         <v>1950</v>
       </c>
-      <c r="C83" s="83"/>
+      <c r="C83" s="85"/>
       <c r="D83" s="77" t="s">
         <v>120</v>
       </c>
@@ -41326,7 +41331,7 @@
       <c r="B84" s="64" t="s">
         <v>1952</v>
       </c>
-      <c r="C84" s="83"/>
+      <c r="C84" s="85"/>
       <c r="D84" s="77" t="s">
         <v>475</v>
       </c>
@@ -41338,7 +41343,7 @@
       <c r="B85" s="64" t="s">
         <v>1954</v>
       </c>
-      <c r="C85" s="83"/>
+      <c r="C85" s="85"/>
       <c r="D85" s="77" t="s">
         <v>23</v>
       </c>
@@ -41350,7 +41355,7 @@
       <c r="B86" s="64" t="s">
         <v>1956</v>
       </c>
-      <c r="C86" s="83"/>
+      <c r="C86" s="85"/>
       <c r="D86" s="77" t="s">
         <v>90</v>
       </c>
@@ -41362,7 +41367,7 @@
       <c r="B87" s="64" t="s">
         <v>1958</v>
       </c>
-      <c r="C87" s="83"/>
+      <c r="C87" s="85"/>
       <c r="D87" s="77" t="s">
         <v>136</v>
       </c>
@@ -41374,7 +41379,7 @@
       <c r="B88" s="64" t="s">
         <v>1960</v>
       </c>
-      <c r="C88" s="83"/>
+      <c r="C88" s="85"/>
       <c r="D88" s="77" t="s">
         <v>152</v>
       </c>
@@ -41386,7 +41391,7 @@
       <c r="B89" s="64" t="s">
         <v>1962</v>
       </c>
-      <c r="C89" s="83"/>
+      <c r="C89" s="85"/>
       <c r="D89" s="77" t="s">
         <v>574</v>
       </c>
@@ -41398,7 +41403,7 @@
       <c r="B90" s="64" t="s">
         <v>1964</v>
       </c>
-      <c r="C90" s="83"/>
+      <c r="C90" s="85"/>
       <c r="D90" s="77" t="s">
         <v>98</v>
       </c>

</xml_diff>

<commit_message>
update del anterior xd
</commit_message>
<xml_diff>
--- a/app/assets/Copia de BASE DE TIENDAS.xlsx
+++ b/app/assets/Copia de BASE DE TIENDAS.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7915944C-D018-46BF-876E-B408E9417B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84C0191E-7361-456C-8653-E023236B09E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8187" uniqueCount="1971">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8190" uniqueCount="1971">
   <si>
     <t>TDA</t>
   </si>
@@ -19787,6 +19787,9 @@
       <c r="G315" t="s">
         <v>1748</v>
       </c>
+      <c r="H315" t="s">
+        <v>1750</v>
+      </c>
       <c r="J315" t="s">
         <v>1749</v>
       </c>
@@ -19819,6 +19822,9 @@
       <c r="G316" t="s">
         <v>1753</v>
       </c>
+      <c r="H316" t="s">
+        <v>1754</v>
+      </c>
       <c r="J316" t="s">
         <v>1749</v>
       </c>
@@ -19850,6 +19856,9 @@
       </c>
       <c r="G317" t="s">
         <v>1757</v>
+      </c>
+      <c r="H317" t="s">
+        <v>1758</v>
       </c>
       <c r="J317" t="s">
         <v>1749</v>

</xml_diff>

<commit_message>
ahora sí quedó la db
</commit_message>
<xml_diff>
--- a/app/assets/Copia de BASE DE TIENDAS.xlsx
+++ b/app/assets/Copia de BASE DE TIENDAS.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84C0191E-7361-456C-8653-E023236B09E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5E82FCB-4AA0-4B19-BCC9-810CA6BBF321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8190" uniqueCount="1971">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8190" uniqueCount="1977">
   <si>
     <t>TDA</t>
   </si>
@@ -5947,6 +5947,24 @@
   </si>
   <si>
     <t>1540112269</t>
+  </si>
+  <si>
+    <t>ameyalli.supervisor@vertiche.com.mx</t>
+  </si>
+  <si>
+    <t>rommel.supervisor@vertiche.com.mx</t>
+  </si>
+  <si>
+    <t>omar.supervisor@vertiche.com.mx</t>
+  </si>
+  <si>
+    <t>a001@vertiche.com.mx</t>
+  </si>
+  <si>
+    <t>r001@vertiche.com.mx</t>
+  </si>
+  <si>
+    <t>o001@vertiche.com.mx</t>
   </si>
 </sst>
 </file>
@@ -5957,7 +5975,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6047,6 +6065,14 @@
       <color theme="1"/>
       <name val="Verdana"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -6297,14 +6323,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="5">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -6527,8 +6554,10 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="5"/>
   </cellXfs>
-  <cellStyles count="5">
+  <cellStyles count="6">
+    <cellStyle name="Hipervínculo" xfId="5" builtinId="8"/>
     <cellStyle name="Moneda 2" xfId="2" xr:uid="{1E95D520-CDC4-4DA1-BDE1-66AF429EA0B0}"/>
     <cellStyle name="Moneda 2 2" xfId="4" xr:uid="{0DF8552F-3C9A-4737-8BCC-871E4A174440}"/>
     <cellStyle name="Moneda 3" xfId="1" xr:uid="{174CF66E-0A5A-46C2-88A0-7FBED3EA6C87}"/>
@@ -19793,14 +19822,14 @@
       <c r="J315" t="s">
         <v>1749</v>
       </c>
-      <c r="K315" t="s">
-        <v>1750</v>
+      <c r="K315" s="86" t="s">
+        <v>1974</v>
       </c>
       <c r="L315" t="s">
         <v>247</v>
       </c>
-      <c r="M315" t="s">
-        <v>1750</v>
+      <c r="M315" s="86" t="s">
+        <v>1971</v>
       </c>
     </row>
     <row r="316" spans="1:13" x14ac:dyDescent="0.3">
@@ -19828,14 +19857,14 @@
       <c r="J316" t="s">
         <v>1749</v>
       </c>
-      <c r="K316" t="s">
-        <v>1754</v>
+      <c r="K316" s="86" t="s">
+        <v>1975</v>
       </c>
       <c r="L316" t="s">
         <v>247</v>
       </c>
-      <c r="M316" t="s">
-        <v>1754</v>
+      <c r="M316" s="86" t="s">
+        <v>1972</v>
       </c>
     </row>
     <row r="317" spans="1:13" x14ac:dyDescent="0.3">
@@ -19863,14 +19892,14 @@
       <c r="J317" t="s">
         <v>1749</v>
       </c>
-      <c r="K317" t="s">
-        <v>1758</v>
+      <c r="K317" s="86" t="s">
+        <v>1976</v>
       </c>
       <c r="L317" t="s">
         <v>247</v>
       </c>
-      <c r="M317" t="s">
-        <v>1758</v>
+      <c r="M317" s="86" t="s">
+        <v>1973</v>
       </c>
     </row>
   </sheetData>
@@ -20178,6 +20207,12 @@
     <hyperlink ref="H314" r:id="rId300" xr:uid="{00000000-0004-0000-0000-00002D010000}"/>
     <hyperlink ref="K314" r:id="rId301" xr:uid="{00000000-0004-0000-0000-00002E010000}"/>
     <hyperlink ref="M70" r:id="rId302" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="M315" r:id="rId303" xr:uid="{DE8F93D2-35FF-48E1-8F9E-D2601F562F5A}"/>
+    <hyperlink ref="M316" r:id="rId304" xr:uid="{12822C1F-054C-4B3B-9CEA-4DAEF8925B81}"/>
+    <hyperlink ref="M317" r:id="rId305" xr:uid="{3976A5D3-C4F8-46E7-83CA-972F79CDBF7D}"/>
+    <hyperlink ref="K315" r:id="rId306" xr:uid="{DF4B9F7E-6386-4E5C-9220-F448C21807BC}"/>
+    <hyperlink ref="K316" r:id="rId307" xr:uid="{36684507-3D64-4919-9F79-C90173F3F572}"/>
+    <hyperlink ref="K317" r:id="rId308" xr:uid="{D41DE9F2-6A86-44F2-AF68-1E7AA7B7590F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>